<commit_message>
v0.17.0: identify map icons and add wiki notes
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/Unidentified_Icons_and_Items.xlsx
+++ b/docs/Unidentified_Icons_and_Items.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Start Here" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Identification list'!$A$1:$I$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Identification list'!$A$1:$I$56</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I94"/>
+  <dimension ref="A1:I56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="34"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -519,37 +519,37 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>U-016</t>
+          <t>U-054</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Misc</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Misc Tab/Misc.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Lower grid C1</t>
+          <t>Shared lower grid R1C1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Purple potion-shaped icon</t>
+          <t>Green face/skull-like emblem on a dark square</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Potion/consumable type unconfirmed.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -562,37 +562,37 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>U-017</t>
+          <t>U-055</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Misc</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Misc Tab/Misc.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Lower grid C2</t>
+          <t>Shared lower grid R1C2</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Purple potion-shaped icon</t>
+          <t>Pale silver folded scroll/leaf-like object</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>223</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Potion/consumable type unconfirmed; large stack. Do not price/vendor by appearance.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -605,27 +605,27 @@
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>U-018</t>
+          <t>U-056</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Gems</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Gems Tab/Gems.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Bottom row R6C1</t>
+          <t>Shared lower grid R1C3</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Dark circular medallion/placeholder icon, red/orange tint; no stack number.</t>
+          <t>Gold circular wheel/star emblem</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -635,7 +635,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Unclear whether this is an owned item, empty-quality placeholder, or UI decoration; exact identity unknown.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -648,27 +648,27 @@
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>U-019</t>
+          <t>U-057</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Gems</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Gems Tab/Gems.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Bottom row R6C2</t>
+          <t>Shared lower grid R1C4</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Dark circular medallion/placeholder icon, purple/magenta tint; no stack number.</t>
+          <t>Blue circular ring/orb</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Unclear whether this is an owned item, empty-quality placeholder, or UI decoration; exact identity unknown.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -691,27 +691,27 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>U-020</t>
+          <t>U-058</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Gems</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Gems Tab/Gems.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Bottom row R6C3</t>
+          <t>Shared lower grid R1C5</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Dark circular medallion/placeholder icon, blue tint; no stack number.</t>
+          <t>Blue-and-gold pointed triangular plaque</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Unclear whether this is an owned item, empty-quality placeholder, or UI decoration; exact identity unknown.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
@@ -734,27 +734,27 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>U-021</t>
+          <t>U-059</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Gems</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Gems Tab/Gems.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Bottom row R6C4</t>
+          <t>Shared lower grid R1C6</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Dark circular medallion/placeholder icon, green tint; no stack number.</t>
+          <t>Gray-blue angular plaque</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Unclear whether this is an owned item, empty-quality placeholder, or UI decoration; exact identity unknown.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
@@ -777,27 +777,27 @@
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>U-022</t>
+          <t>U-060</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Gems</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Gems Tab/Gems.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Bottom row R6C5</t>
+          <t>Shared lower grid R1C7</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Dark circular medallion/placeholder icon, gold/yellow tint; no stack number.</t>
+          <t>Blue-gray angular plaque</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -807,7 +807,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Unclear whether this is an owned item, empty-quality placeholder, or UI decoration; exact identity unknown.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
@@ -820,27 +820,27 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>U-023</t>
+          <t>U-061</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Gems</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Gems Tab/Gems.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Bottom row R6C6</t>
+          <t>Shared lower grid R2C1</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Dark circular medallion/placeholder icon, gray/silver tint; no stack number.</t>
+          <t>Cream/green map or medallion with a blue mark</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Unclear whether this is an owned item, empty-quality placeholder, or UI decoration; exact identity unknown.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -863,27 +863,27 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>U-024</t>
+          <t>U-062</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Gems</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Gems Tab/Gems.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Bottom row R6C7</t>
+          <t>Shared lower grid R2C2</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Dark circular medallion/placeholder icon, skull/white tint; no stack number.</t>
+          <t>Pale beige circular lens/orb</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Unclear whether this is an owned item, empty-quality placeholder, or UI decoration; exact identity unknown.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
@@ -906,37 +906,37 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>U-025</t>
+          <t>U-063</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C1</t>
+          <t>Shared lower grid R2C3</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: green/cream diamond emblem</t>
+          <t>Round red/yellow segmented emblem</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -949,37 +949,37 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>U-026</t>
+          <t>U-064</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C2</t>
+          <t>Shared lower grid R2C4</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: red/brown angular emblem</t>
+          <t>Small blue-gray circular object</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -992,37 +992,37 @@
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>U-027</t>
+          <t>U-065</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C3</t>
+          <t>Shared lower grid R2C5</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: green/red emblem</t>
+          <t>Blue/gold polygonal plaque</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -1035,37 +1035,37 @@
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>U-028</t>
+          <t>U-066</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C4</t>
+          <t>Shared lower grid R2C6</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: tan/olive emblem</t>
+          <t>Pale silver folded card/scroll</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
@@ -1078,37 +1078,37 @@
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>U-029</t>
+          <t>U-067</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C5</t>
+          <t>Shared lower grid R2C7</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: purple/green emblem</t>
+          <t>Yellow-gray ornate block/emblem</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
@@ -1121,37 +1121,37 @@
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>U-030</t>
+          <t>U-068</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C6</t>
+          <t>Shared lower grid R3C1</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: blue/teal emblem</t>
+          <t>Brown oval spiral/relic icon</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr"/>
@@ -1164,37 +1164,37 @@
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>U-031</t>
+          <t>U-069</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C7</t>
+          <t>Shared lower grid R3C2</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: red/yellow emblem</t>
+          <t>Dark brown/red ring-shaped relic</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
@@ -1207,37 +1207,37 @@
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>U-032</t>
+          <t>U-070</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C8</t>
+          <t>Shared lower grid R3C3</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: orange/gray emblem</t>
+          <t>Bronze-brown ring/loop icon</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
@@ -1250,37 +1250,37 @@
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>U-033</t>
+          <t>U-071</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C9</t>
+          <t>Shared lower grid R3C4</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: yellow/green emblem</t>
+          <t>Tan folded scroll/loop icon</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
@@ -1293,37 +1293,37 @@
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>U-034</t>
+          <t>U-072</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 1</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R2C1</t>
+          <t>Shared lower grid R3C5</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: green/cream emblem</t>
+          <t>Pale brown curved ring/relic</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
@@ -1336,37 +1336,37 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>U-035</t>
+          <t>U-073</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C1</t>
+          <t>Shared lower grid R3C6</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: blue/gray star emblem</t>
+          <t>Brown oval ring/relic</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
@@ -1379,37 +1379,37 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>U-036</t>
+          <t>U-074</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Maps, shared lower grid</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C2</t>
+          <t>Shared lower grid R3C7</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: teal/green emblem</t>
+          <t>Brown spiral/loop relic</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No number visible</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>
@@ -1422,37 +1422,37 @@
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>U-037</t>
+          <t>U-075</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C3</t>
+          <t>R1C1</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: cream/red/yellow emblem</t>
+          <t>Round-headed brown wand/key-like icon</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr"/>
@@ -1465,37 +1465,37 @@
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>U-038</t>
+          <t>U-076</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C4</t>
+          <t>R1C2</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: dark gray emblem</t>
+          <t>Round-headed gold wand/key-like icon</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr"/>
@@ -1508,37 +1508,37 @@
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>U-039</t>
+          <t>U-077</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C5</t>
+          <t>R1C3</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: blue/gray emblem</t>
+          <t>Round-headed gray wand/key-like icon</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr"/>
@@ -1551,37 +1551,37 @@
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>U-040</t>
+          <t>U-078</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C6</t>
+          <t>R2C1</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: gold/orange emblem</t>
+          <t>Vertical brown key-shaped icon</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr"/>
@@ -1594,37 +1594,37 @@
     <row r="27" ht="42" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>U-041</t>
+          <t>U-079</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C7</t>
+          <t>R2C2</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: gray/teal emblem</t>
+          <t>Vertical gold key-shaped icon</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr"/>
@@ -1637,37 +1637,37 @@
     <row r="28" ht="42" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>U-042</t>
+          <t>U-080</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C8</t>
+          <t>R2C3</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: red/black emblem</t>
+          <t>Vertical silver key-shaped icon</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr"/>
@@ -1680,37 +1680,37 @@
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>U-043</t>
+          <t>U-081</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C9</t>
+          <t>R3C1</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: teal/gray emblem</t>
+          <t>Brown mottled oval/organ-like icon</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr"/>
@@ -1723,37 +1723,37 @@
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>U-044</t>
+          <t>U-082</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 2</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 2 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R2C1</t>
+          <t>R3C2</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: red/orange emblem</t>
+          <t>Pale circular eye-like icon with red markings</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
@@ -1766,37 +1766,37 @@
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>U-045</t>
+          <t>U-083</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C1</t>
+          <t>R3C3</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: blue/purple star emblem</t>
+          <t>Narrow pale curved/blade-like icon</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -1809,37 +1809,37 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>U-046</t>
+          <t>U-084</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C2</t>
+          <t>R4C2</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: green/tan emblem</t>
+          <t>Pale green circular medallion with geometric symbol</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
@@ -1852,37 +1852,37 @@
     <row r="33" ht="42" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>U-047</t>
+          <t>U-085</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C3</t>
+          <t>R1C1</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: red/orange star emblem</t>
+          <t>Gray hexagonal emblem</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -1895,37 +1895,37 @@
     <row r="34" ht="42" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>U-048</t>
+          <t>U-086</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C4</t>
+          <t>R1C2</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: brown/red star emblem</t>
+          <t>Red angular object</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
@@ -1938,37 +1938,37 @@
     <row r="35" ht="42" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>U-049</t>
+          <t>U-087</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C5</t>
+          <t>R1C3</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: blue/gold emblem</t>
+          <t>White curved item; a white “1” overlay is visible</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>R1C3 has visible “1”; meaning unconfirmed</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr"/>
@@ -1981,37 +1981,37 @@
     <row r="36" ht="42" customHeight="1">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>U-050</t>
+          <t>U-088</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C6</t>
+          <t>R1C4</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: gray/blue emblem</t>
+          <t>Red triangle/rune-like icon</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H36" s="3" t="inlineStr"/>
@@ -2024,37 +2024,37 @@
     <row r="37" ht="42" customHeight="1">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>U-051</t>
+          <t>U-089</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C7</t>
+          <t>R2C1</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: green/orange emblem</t>
+          <t>Gold/red plate-like icon</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H37" s="3" t="inlineStr"/>
@@ -2067,37 +2067,37 @@
     <row r="38" ht="42" customHeight="1">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>U-052</t>
+          <t>U-090</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C8</t>
+          <t>R2C2</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: red/orange emblem</t>
+          <t>Red orb</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H38" s="3" t="inlineStr"/>
@@ -2110,37 +2110,37 @@
     <row r="39" ht="42" customHeight="1">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>U-053</t>
+          <t>U-091</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, Tier 3</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 3 - No Maps.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Top map-like grid R1C9</t>
+          <t>R2C3</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Small square banner/tile: teal/rust emblem</t>
+          <t>Blue pointed shard</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>No stack number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Source filename says “No Maps”; no tooltip/ownership indicator. Could be UI map slots rather than owned items; please confirm.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr"/>
@@ -2153,37 +2153,37 @@
     <row r="40" ht="42" customHeight="1">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>U-054</t>
+          <t>U-092</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C1</t>
+          <t>R2C4</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Green face/skull-like emblem on a dark square</t>
+          <t>Red hand/wing-like icon</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr"/>
@@ -2196,37 +2196,37 @@
     <row r="41" ht="42" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>U-055</t>
+          <t>U-093</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C2</t>
+          <t>R3C1</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Pale silver folded scroll/leaf-like object</t>
+          <t>Blue rune/plate-like icon</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr"/>
@@ -2239,37 +2239,37 @@
     <row r="42" ht="42" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>U-056</t>
+          <t>U-094</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C3</t>
+          <t>R3C2</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Gold circular wheel/star emblem</t>
+          <t>Dark red shard</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr"/>
@@ -2282,37 +2282,37 @@
     <row r="43" ht="42" customHeight="1">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>U-057</t>
+          <t>U-095</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C4</t>
+          <t>R3C3</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Blue circular ring/orb</t>
+          <t>Flame-shaped icon</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr"/>
@@ -2325,37 +2325,37 @@
     <row r="44" ht="42" customHeight="1">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>U-058</t>
+          <t>U-096</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C5</t>
+          <t>R3C4</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Blue-and-gold pointed triangular plaque</t>
+          <t>Dark framed tablet/book-like icon</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr"/>
@@ -2368,37 +2368,37 @@
     <row r="45" ht="42" customHeight="1">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>U-059</t>
+          <t>U-097</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C6</t>
+          <t>R4C1</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Gray-blue angular plaque</t>
+          <t>Multi-stone emblem</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr"/>
@@ -2411,37 +2411,37 @@
     <row r="46" ht="42" customHeight="1">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>U-060</t>
+          <t>U-098</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C7</t>
+          <t>R4C2</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Blue-gray angular plaque</t>
+          <t>Red orb</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr"/>
@@ -2454,37 +2454,37 @@
     <row r="47" ht="42" customHeight="1">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>U-061</t>
+          <t>U-099</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C1</t>
+          <t>R4C3</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Cream/green map or medallion with a blue mark</t>
+          <t>Blue orb</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H47" s="3" t="inlineStr"/>
@@ -2497,37 +2497,37 @@
     <row r="48" ht="42" customHeight="1">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>U-062</t>
+          <t>U-100</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C2</t>
+          <t>R4C4</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Pale beige circular lens/orb</t>
+          <t>Brown spiral/swirl icon</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H48" s="3" t="inlineStr"/>
@@ -2540,37 +2540,37 @@
     <row r="49" ht="42" customHeight="1">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>U-063</t>
+          <t>U-101</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C3</t>
+          <t>Top-centre crossed-axe icon</t>
         </is>
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Round red/yellow segmented emblem</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>14 points</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Previously read as possibly Double Swing or Double Throw; confirm exact skill name.</t>
         </is>
       </c>
       <c r="H49" s="3" t="inlineStr"/>
@@ -2583,37 +2583,37 @@
     <row r="50" ht="42" customHeight="1">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>U-064</t>
+          <t>U-102</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C4</t>
+          <t>Upper-right node</t>
         </is>
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Small blue-gray circular object</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>21 points</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Skill name was not confirmed from tooltip.</t>
         </is>
       </c>
       <c r="H50" s="3" t="inlineStr"/>
@@ -2626,37 +2626,37 @@
     <row r="51" ht="42" customHeight="1">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>U-065</t>
+          <t>U-103</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C5</t>
+          <t>Mid-right node</t>
         </is>
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Blue/gold polygonal plaque</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>21 points</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Skill name was not confirmed from tooltip.</t>
         </is>
       </c>
       <c r="H51" s="3" t="inlineStr"/>
@@ -2669,37 +2669,37 @@
     <row r="52" ht="42" customHeight="1">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>U-066</t>
+          <t>U-104</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C6</t>
+          <t>Prerequisite path / lower nodes</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Pale silver folded card/scroll</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>Several nodes show 2 points</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Prior summary did not preserve exact coordinates/names for every 2-point node; identify if useful.</t>
         </is>
       </c>
       <c r="H52" s="3" t="inlineStr"/>
@@ -2712,37 +2712,37 @@
     <row r="53" ht="42" customHeight="1">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>U-067</t>
+          <t>U-105</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Combat Masteries</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C7</t>
+          <t>Top-right thrown-weapon icon</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Yellow-gray ornate block/emblem</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>21 points</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Previously inferred as Throw Mastery; confirm exact label.</t>
         </is>
       </c>
       <c r="H53" s="3" t="inlineStr"/>
@@ -2755,37 +2755,37 @@
     <row r="54" ht="42" customHeight="1">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>U-068</t>
+          <t>U-106</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Combat Masteries</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C1</t>
+          <t>Left-mid, right-mid, bottom-left, bottom-right nodes</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Brown oval spiral/relic icon</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>2 points each</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Skill names not confirmed by hover labels.</t>
         </is>
       </c>
       <c r="H54" s="3" t="inlineStr"/>
@@ -2798,37 +2798,37 @@
     <row r="55" ht="42" customHeight="1">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>U-069</t>
+          <t>U-107</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Warcries</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C2</t>
+          <t>Top-right node</t>
         </is>
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Dark brown/red ring-shaped relic</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>4 points</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Previously inferred as Battle Command; confirm exact label.</t>
         </is>
       </c>
       <c r="H55" s="3" t="inlineStr"/>
@@ -2841,37 +2841,37 @@
     <row r="56" ht="42" customHeight="1">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>U-070</t>
+          <t>U-108</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Character — Warcries</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C3</t>
+          <t>Left-side node path</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Bronze-brown ring/loop icon</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>Four nodes show 2 points each</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>Previously summarized as the Battle Orders/Shout/Find Potion path; exact names/positions need confirmation.</t>
         </is>
       </c>
       <c r="H56" s="3" t="inlineStr"/>
@@ -2881,1640 +2881,44 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="42" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>U-071</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Maps, shared lower grid</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
-        </is>
-      </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Shared lower grid R3C4</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>Tan folded scroll/loop icon</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>No number visible</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="inlineStr">
-        <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
-        </is>
-      </c>
-      <c r="H57" s="3" t="inlineStr"/>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="42" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>U-072</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Maps, shared lower grid</t>
-        </is>
-      </c>
-      <c r="C58" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="inlineStr">
-        <is>
-          <t>Shared lower grid R3C5</t>
-        </is>
-      </c>
-      <c r="E58" s="2" t="inlineStr">
-        <is>
-          <t>Pale brown curved ring/relic</t>
-        </is>
-      </c>
-      <c r="F58" s="2" t="inlineStr">
-        <is>
-          <t>No number visible</t>
-        </is>
-      </c>
-      <c r="G58" s="2" t="inlineStr">
-        <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
-        </is>
-      </c>
-      <c r="H58" s="3" t="inlineStr"/>
-      <c r="I58" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="42" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>U-073</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Maps, shared lower grid</t>
-        </is>
-      </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Shared lower grid R3C6</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>Brown oval ring/relic</t>
-        </is>
-      </c>
-      <c r="F59" s="2" t="inlineStr">
-        <is>
-          <t>No number visible</t>
-        </is>
-      </c>
-      <c r="G59" s="2" t="inlineStr">
-        <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
-        </is>
-      </c>
-      <c r="H59" s="3" t="inlineStr"/>
-      <c r="I59" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="42" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>U-074</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Maps, shared lower grid</t>
-        </is>
-      </c>
-      <c r="C60" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
-        </is>
-      </c>
-      <c r="D60" s="2" t="inlineStr">
-        <is>
-          <t>Shared lower grid R3C7</t>
-        </is>
-      </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Brown spiral/loop relic</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="inlineStr">
-        <is>
-          <t>No number visible</t>
-        </is>
-      </c>
-      <c r="G60" s="2" t="inlineStr">
-        <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
-        </is>
-      </c>
-      <c r="H60" s="3" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="42" customHeight="1">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>U-075</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C61" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D61" s="2" t="inlineStr">
-        <is>
-          <t>R1C1</t>
-        </is>
-      </c>
-      <c r="E61" s="2" t="inlineStr">
-        <is>
-          <t>Round-headed brown wand/key-like icon</t>
-        </is>
-      </c>
-      <c r="F61" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G61" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H61" s="3" t="inlineStr"/>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="42" customHeight="1">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>U-076</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>R1C2</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>Round-headed gold wand/key-like icon</t>
-        </is>
-      </c>
-      <c r="F62" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H62" s="3" t="inlineStr"/>
-      <c r="I62" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="42" customHeight="1">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>U-077</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>R1C3</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>Round-headed gray wand/key-like icon</t>
-        </is>
-      </c>
-      <c r="F63" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H63" s="3" t="inlineStr"/>
-      <c r="I63" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="42" customHeight="1">
-      <c r="A64" s="2" t="inlineStr">
-        <is>
-          <t>U-078</t>
-        </is>
-      </c>
-      <c r="B64" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>R2C1</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>Vertical brown key-shaped icon</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H64" s="3" t="inlineStr"/>
-      <c r="I64" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="42" customHeight="1">
-      <c r="A65" s="2" t="inlineStr">
-        <is>
-          <t>U-079</t>
-        </is>
-      </c>
-      <c r="B65" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C65" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D65" s="2" t="inlineStr">
-        <is>
-          <t>R2C2</t>
-        </is>
-      </c>
-      <c r="E65" s="2" t="inlineStr">
-        <is>
-          <t>Vertical gold key-shaped icon</t>
-        </is>
-      </c>
-      <c r="F65" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G65" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H65" s="3" t="inlineStr"/>
-      <c r="I65" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="42" customHeight="1">
-      <c r="A66" s="2" t="inlineStr">
-        <is>
-          <t>U-080</t>
-        </is>
-      </c>
-      <c r="B66" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C66" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>R2C3</t>
-        </is>
-      </c>
-      <c r="E66" s="2" t="inlineStr">
-        <is>
-          <t>Vertical silver key-shaped icon</t>
-        </is>
-      </c>
-      <c r="F66" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G66" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H66" s="3" t="inlineStr"/>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="42" customHeight="1">
-      <c r="A67" s="2" t="inlineStr">
-        <is>
-          <t>U-081</t>
-        </is>
-      </c>
-      <c r="B67" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C67" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D67" s="2" t="inlineStr">
-        <is>
-          <t>R3C1</t>
-        </is>
-      </c>
-      <c r="E67" s="2" t="inlineStr">
-        <is>
-          <t>Brown mottled oval/organ-like icon</t>
-        </is>
-      </c>
-      <c r="F67" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G67" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H67" s="3" t="inlineStr"/>
-      <c r="I67" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="42" customHeight="1">
-      <c r="A68" s="2" t="inlineStr">
-        <is>
-          <t>U-082</t>
-        </is>
-      </c>
-      <c r="B68" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C68" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D68" s="2" t="inlineStr">
-        <is>
-          <t>R3C2</t>
-        </is>
-      </c>
-      <c r="E68" s="2" t="inlineStr">
-        <is>
-          <t>Pale circular eye-like icon with red markings</t>
-        </is>
-      </c>
-      <c r="F68" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G68" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H68" s="3" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="42" customHeight="1">
-      <c r="A69" s="2" t="inlineStr">
-        <is>
-          <t>U-083</t>
-        </is>
-      </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C69" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="inlineStr">
-        <is>
-          <t>R3C3</t>
-        </is>
-      </c>
-      <c r="E69" s="2" t="inlineStr">
-        <is>
-          <t>Narrow pale curved/blade-like icon</t>
-        </is>
-      </c>
-      <c r="F69" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G69" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H69" s="3" t="inlineStr"/>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="42" customHeight="1">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>U-084</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (left grid)</t>
-        </is>
-      </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>R4C2</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Pale green circular medallion with geometric symbol</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H70" s="3" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="42" customHeight="1">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>U-085</t>
-        </is>
-      </c>
-      <c r="B71" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C71" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D71" s="2" t="inlineStr">
-        <is>
-          <t>R1C1</t>
-        </is>
-      </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>Gray hexagonal emblem</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H71" s="3" t="inlineStr"/>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="42" customHeight="1">
-      <c r="A72" s="2" t="inlineStr">
-        <is>
-          <t>U-086</t>
-        </is>
-      </c>
-      <c r="B72" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C72" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D72" s="2" t="inlineStr">
-        <is>
-          <t>R1C2</t>
-        </is>
-      </c>
-      <c r="E72" s="2" t="inlineStr">
-        <is>
-          <t>Red angular object</t>
-        </is>
-      </c>
-      <c r="F72" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G72" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H72" s="3" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="42" customHeight="1">
-      <c r="A73" s="2" t="inlineStr">
-        <is>
-          <t>U-087</t>
-        </is>
-      </c>
-      <c r="B73" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C73" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D73" s="2" t="inlineStr">
-        <is>
-          <t>R1C3</t>
-        </is>
-      </c>
-      <c r="E73" s="2" t="inlineStr">
-        <is>
-          <t>White curved item; a white “1” overlay is visible</t>
-        </is>
-      </c>
-      <c r="F73" s="2" t="inlineStr">
-        <is>
-          <t>R1C3 has visible “1”; meaning unconfirmed</t>
-        </is>
-      </c>
-      <c r="G73" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H73" s="3" t="inlineStr"/>
-      <c r="I73" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="42" customHeight="1">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>U-088</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>R1C4</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>Red triangle/rune-like icon</t>
-        </is>
-      </c>
-      <c r="F74" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G74" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H74" s="3" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="42" customHeight="1">
-      <c r="A75" s="2" t="inlineStr">
-        <is>
-          <t>U-089</t>
-        </is>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="inlineStr">
-        <is>
-          <t>R2C1</t>
-        </is>
-      </c>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Gold/red plate-like icon</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H75" s="3" t="inlineStr"/>
-      <c r="I75" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="42" customHeight="1">
-      <c r="A76" s="2" t="inlineStr">
-        <is>
-          <t>U-090</t>
-        </is>
-      </c>
-      <c r="B76" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C76" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D76" s="2" t="inlineStr">
-        <is>
-          <t>R2C2</t>
-        </is>
-      </c>
-      <c r="E76" s="2" t="inlineStr">
-        <is>
-          <t>Red orb</t>
-        </is>
-      </c>
-      <c r="F76" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G76" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H76" s="3" t="inlineStr"/>
-      <c r="I76" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="42" customHeight="1">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>U-091</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>R2C3</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>Blue pointed shard</t>
-        </is>
-      </c>
-      <c r="F77" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G77" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H77" s="3" t="inlineStr"/>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="42" customHeight="1">
-      <c r="A78" s="2" t="inlineStr">
-        <is>
-          <t>U-092</t>
-        </is>
-      </c>
-      <c r="B78" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C78" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D78" s="2" t="inlineStr">
-        <is>
-          <t>R2C4</t>
-        </is>
-      </c>
-      <c r="E78" s="2" t="inlineStr">
-        <is>
-          <t>Red hand/wing-like icon</t>
-        </is>
-      </c>
-      <c r="F78" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G78" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H78" s="3" t="inlineStr"/>
-      <c r="I78" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="42" customHeight="1">
-      <c r="A79" s="2" t="inlineStr">
-        <is>
-          <t>U-093</t>
-        </is>
-      </c>
-      <c r="B79" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C79" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D79" s="2" t="inlineStr">
-        <is>
-          <t>R3C1</t>
-        </is>
-      </c>
-      <c r="E79" s="2" t="inlineStr">
-        <is>
-          <t>Blue rune/plate-like icon</t>
-        </is>
-      </c>
-      <c r="F79" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G79" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H79" s="3" t="inlineStr"/>
-      <c r="I79" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="42" customHeight="1">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>U-094</t>
-        </is>
-      </c>
-      <c r="B80" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C80" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D80" s="2" t="inlineStr">
-        <is>
-          <t>R3C2</t>
-        </is>
-      </c>
-      <c r="E80" s="2" t="inlineStr">
-        <is>
-          <t>Dark red shard</t>
-        </is>
-      </c>
-      <c r="F80" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G80" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H80" s="3" t="inlineStr"/>
-      <c r="I80" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="42" customHeight="1">
-      <c r="A81" s="2" t="inlineStr">
-        <is>
-          <t>U-095</t>
-        </is>
-      </c>
-      <c r="B81" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
-        <is>
-          <t>R3C3</t>
-        </is>
-      </c>
-      <c r="E81" s="2" t="inlineStr">
-        <is>
-          <t>Flame-shaped icon</t>
-        </is>
-      </c>
-      <c r="F81" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G81" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H81" s="3" t="inlineStr"/>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="42" customHeight="1">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>U-096</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>R3C4</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>Dark framed tablet/book-like icon</t>
-        </is>
-      </c>
-      <c r="F82" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G82" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H82" s="3" t="inlineStr"/>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="42" customHeight="1">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>U-097</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
-        <is>
-          <t>R4C1</t>
-        </is>
-      </c>
-      <c r="E83" s="2" t="inlineStr">
-        <is>
-          <t>Multi-stone emblem</t>
-        </is>
-      </c>
-      <c r="F83" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G83" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H83" s="3" t="inlineStr"/>
-      <c r="I83" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="42" customHeight="1">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>U-098</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>R4C2</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>Red orb</t>
-        </is>
-      </c>
-      <c r="F84" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G84" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H84" s="3" t="inlineStr"/>
-      <c r="I84" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="42" customHeight="1">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>U-099</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>R4C3</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>Blue orb</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G85" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H85" s="3" t="inlineStr"/>
-      <c r="I85" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="42" customHeight="1">
-      <c r="A86" s="2" t="inlineStr">
-        <is>
-          <t>U-100</t>
-        </is>
-      </c>
-      <c r="B86" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
-        <is>
-          <t>R4C4</t>
-        </is>
-      </c>
-      <c r="E86" s="2" t="inlineStr">
-        <is>
-          <t>Brown spiral/swirl icon</t>
-        </is>
-      </c>
-      <c r="F86" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G86" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H86" s="3" t="inlineStr"/>
-      <c r="I86" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="42" customHeight="1">
-      <c r="A87" s="2" t="inlineStr">
-        <is>
-          <t>U-101</t>
-        </is>
-      </c>
-      <c r="B87" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
-        <is>
-          <t>Top-centre crossed-axe icon</t>
-        </is>
-      </c>
-      <c r="E87" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F87" s="2" t="inlineStr">
-        <is>
-          <t>14 points</t>
-        </is>
-      </c>
-      <c r="G87" s="2" t="inlineStr">
-        <is>
-          <t>Previously read as possibly Double Swing or Double Throw; confirm exact skill name.</t>
-        </is>
-      </c>
-      <c r="H87" s="3" t="inlineStr"/>
-      <c r="I87" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="42" customHeight="1">
-      <c r="A88" s="2" t="inlineStr">
-        <is>
-          <t>U-102</t>
-        </is>
-      </c>
-      <c r="B88" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>Upper-right node</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>21 points</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>Skill name was not confirmed from tooltip.</t>
-        </is>
-      </c>
-      <c r="H88" s="3" t="inlineStr"/>
-      <c r="I88" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="42" customHeight="1">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>U-103</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>Mid-right node</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F89" s="2" t="inlineStr">
-        <is>
-          <t>21 points</t>
-        </is>
-      </c>
-      <c r="G89" s="2" t="inlineStr">
-        <is>
-          <t>Skill name was not confirmed from tooltip.</t>
-        </is>
-      </c>
-      <c r="H89" s="3" t="inlineStr"/>
-      <c r="I89" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="42" customHeight="1">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>U-104</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>Prerequisite path / lower nodes</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>Several nodes show 2 points</t>
-        </is>
-      </c>
-      <c r="G90" s="2" t="inlineStr">
-        <is>
-          <t>Prior summary did not preserve exact coordinates/names for every 2-point node; identify if useful.</t>
-        </is>
-      </c>
-      <c r="H90" s="3" t="inlineStr"/>
-      <c r="I90" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="42" customHeight="1">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>U-105</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Masteries</t>
-        </is>
-      </c>
-      <c r="C91" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
-        </is>
-      </c>
-      <c r="D91" s="2" t="inlineStr">
-        <is>
-          <t>Top-right thrown-weapon icon</t>
-        </is>
-      </c>
-      <c r="E91" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F91" s="2" t="inlineStr">
-        <is>
-          <t>21 points</t>
-        </is>
-      </c>
-      <c r="G91" s="2" t="inlineStr">
-        <is>
-          <t>Previously inferred as Throw Mastery; confirm exact label.</t>
-        </is>
-      </c>
-      <c r="H91" s="3" t="inlineStr"/>
-      <c r="I91" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="42" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>U-106</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Masteries</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>Left-mid, right-mid, bottom-left, bottom-right nodes</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>2 points each</t>
-        </is>
-      </c>
-      <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>Skill names not confirmed by hover labels.</t>
-        </is>
-      </c>
-      <c r="H92" s="3" t="inlineStr"/>
-      <c r="I92" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="42" customHeight="1">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>U-107</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
-        <is>
-          <t>Character — Warcries</t>
-        </is>
-      </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>Top-right node</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F93" s="2" t="inlineStr">
-        <is>
-          <t>4 points</t>
-        </is>
-      </c>
-      <c r="G93" s="2" t="inlineStr">
-        <is>
-          <t>Previously inferred as Battle Command; confirm exact label.</t>
-        </is>
-      </c>
-      <c r="H93" s="3" t="inlineStr"/>
-      <c r="I93" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="42" customHeight="1">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>U-108</t>
-        </is>
-      </c>
-      <c r="B94" s="2" t="inlineStr">
-        <is>
-          <t>Character — Warcries</t>
-        </is>
-      </c>
-      <c r="C94" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
-        </is>
-      </c>
-      <c r="D94" s="2" t="inlineStr">
-        <is>
-          <t>Left-side node path</t>
-        </is>
-      </c>
-      <c r="E94" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>Four nodes show 2 points each</t>
-        </is>
-      </c>
-      <c r="G94" s="2" t="inlineStr">
-        <is>
-          <t>Previously summarized as the Battle Orders/Shout/Find Potion path; exact names/positions need confirmation.</t>
-        </is>
-      </c>
-      <c r="H94" s="3" t="inlineStr"/>
-      <c r="I94" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
+    <row r="57" ht="42" customHeight="1"/>
+    <row r="58" ht="42" customHeight="1"/>
+    <row r="59" ht="42" customHeight="1"/>
+    <row r="60" ht="42" customHeight="1"/>
+    <row r="61" ht="42" customHeight="1"/>
+    <row r="62" ht="42" customHeight="1"/>
+    <row r="63" ht="42" customHeight="1"/>
+    <row r="64" ht="42" customHeight="1"/>
+    <row r="65" ht="42" customHeight="1"/>
+    <row r="66" ht="42" customHeight="1"/>
+    <row r="67" ht="42" customHeight="1"/>
+    <row r="68" ht="42" customHeight="1"/>
+    <row r="69" ht="42" customHeight="1"/>
+    <row r="70" ht="42" customHeight="1"/>
+    <row r="71" ht="42" customHeight="1"/>
+    <row r="72" ht="42" customHeight="1"/>
+    <row r="73" ht="42" customHeight="1"/>
+    <row r="74" ht="42" customHeight="1"/>
+    <row r="75" ht="42" customHeight="1"/>
+    <row r="76" ht="42" customHeight="1"/>
+    <row r="77" ht="42" customHeight="1"/>
+    <row r="78" ht="42" customHeight="1"/>
+    <row r="79" ht="42" customHeight="1"/>
+    <row r="80" ht="42" customHeight="1"/>
+    <row r="81" ht="42" customHeight="1"/>
+    <row r="82" ht="42" customHeight="1"/>
+    <row r="83" ht="42" customHeight="1"/>
+    <row r="84" ht="42" customHeight="1"/>
+    <row r="85" ht="42" customHeight="1"/>
+    <row r="86" ht="42" customHeight="1"/>
+    <row r="87" ht="42" customHeight="1"/>
+    <row r="88" ht="42" customHeight="1"/>
+    <row r="89" ht="42" customHeight="1"/>
+    <row r="90" ht="42" customHeight="1"/>
+    <row r="91" ht="42" customHeight="1"/>
+    <row r="92" ht="42" customHeight="1"/>
+    <row r="93" ht="42" customHeight="1"/>
+    <row r="94" ht="42" customHeight="1"/>
     <row r="95" ht="42" customHeight="1"/>
     <row r="96" ht="42" customHeight="1"/>
     <row r="97" ht="42" customHeight="1"/>
@@ -4531,7 +2935,7 @@
     <row r="108" ht="42" customHeight="1"/>
     <row r="109" ht="42" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:I94"/>
+  <autoFilter ref="A1:I56"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4542,7 +2946,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="34"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -4589,7 +2993,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>93 unresolved rows: 85 inventory-related icons/slots + 8 skill-tree name checks. U-001–U-015 are resolved and recorded in docs/04D_Inventory_Misc.md.</t>
+          <t>55 unresolved rows: 47 inventory/UI icons + 8 skill-tree name checks. U-001–U-053 are resolved and recorded in source documents.</t>
         </is>
       </c>
     </row>
@@ -4601,7 +3005,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Misc: 2 remaining; Gems bottom row: 7; Maps tier tiles: 29; Maps shared lower grid: 21; Ubers: 26; skill-tree checks: 8.</t>
+          <t>Misc: 0; Gems bottom row: 0; Maps top tiles: 0 (names/wiki notes recorded); Maps shared lower grid: 21; Ubers: 26; skill-tree checks: 8.</t>
         </is>
       </c>
     </row>
@@ -4613,7 +3017,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Map screenshots say “No Maps”; the 29 top tiles may be UI/map-category slots rather than owned items. Lower grid repeats in all three screenshots and is counted once.</t>
+          <t>Top map icons are named, but the source screenshots say “No Maps” and do not confirm map ownership. The repeated lower 3×7 grid remains unidentified.</t>
         </is>
       </c>
     </row>
@@ -4661,7 +3065,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>When you finish entering descriptions, tell me or upload/save the completed workbook. I will use your descriptions to resolve the corresponding image records before producing final swap/keep/sell/trade recommendations.</t>
+          <t>Player will upload identification updates after every 20 lines. Fill “Your identification / description” for remaining rows; I will update the relevant docs and remove completed IDs from this tracker.</t>
         </is>
       </c>
     </row>
@@ -4685,7 +3089,19 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>U-001 through U-015 identified in docs/1-15 Identified.xlsx; transcribed to docs/04D_Inventory_Misc.md and removed from the unresolved list.</t>
+          <t>U-001–U-015 and U-016–U-053 are resolved and documented; see docs/04D_Inventory_Misc.md, docs/04F_Inventory_Gems.md, and docs/04I_Inventory_Maps.md. Source uploads remain in docs/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Wiki lookup</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Targeted Maps page lookup completed for U-035–U-053; broader PD2 Wiki review remains deferred until all identifications are complete.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document map item IDs U-054 to U-074
Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/Unidentified_Icons_and_Items.xlsx
+++ b/docs/Unidentified_Icons_and_Items.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Start Here" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Identification list'!$A$1:$I$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Identification list'!$A$1:$I$35</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I56"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="34"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -519,37 +519,37 @@
     <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>U-054</t>
+          <t>U-075</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C1</t>
+          <t>R1C1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Green face/skull-like emblem on a dark square</t>
+          <t>Round-headed brown wand/key-like icon</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr"/>
@@ -562,37 +562,37 @@
     <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>U-055</t>
+          <t>U-076</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C2</t>
+          <t>R1C2</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Pale silver folded scroll/leaf-like object</t>
+          <t>Round-headed gold wand/key-like icon</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr"/>
@@ -605,37 +605,37 @@
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>U-056</t>
+          <t>U-077</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C3</t>
+          <t>R1C3</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Gold circular wheel/star emblem</t>
+          <t>Round-headed gray wand/key-like icon</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr"/>
@@ -648,37 +648,37 @@
     <row r="5" ht="42" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>U-057</t>
+          <t>U-078</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C4</t>
+          <t>R2C1</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Blue circular ring/orb</t>
+          <t>Vertical brown key-shaped icon</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr"/>
@@ -691,37 +691,37 @@
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>U-058</t>
+          <t>U-079</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C5</t>
+          <t>R2C2</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Blue-and-gold pointed triangular plaque</t>
+          <t>Vertical gold key-shaped icon</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr"/>
@@ -734,37 +734,37 @@
     <row r="7" ht="42" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>U-059</t>
+          <t>U-080</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C6</t>
+          <t>R2C3</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Gray-blue angular plaque</t>
+          <t>Vertical silver key-shaped icon</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr"/>
@@ -777,37 +777,37 @@
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>U-060</t>
+          <t>U-081</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R1C7</t>
+          <t>R3C1</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Blue-gray angular plaque</t>
+          <t>Brown mottled oval/organ-like icon</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr"/>
@@ -820,37 +820,37 @@
     <row r="9" ht="42" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>U-061</t>
+          <t>U-082</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C1</t>
+          <t>R3C2</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Cream/green map or medallion with a blue mark</t>
+          <t>Pale circular eye-like icon with red markings</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr"/>
@@ -863,37 +863,37 @@
     <row r="10" ht="42" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>U-062</t>
+          <t>U-083</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C2</t>
+          <t>R3C3</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Pale beige circular lens/orb</t>
+          <t>Narrow pale curved/blade-like icon</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr"/>
@@ -906,37 +906,37 @@
     <row r="11" ht="42" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>U-063</t>
+          <t>U-084</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (left grid)</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C3</t>
+          <t>R4C2</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Round red/yellow segmented emblem</t>
+          <t>Pale green circular medallion with geometric symbol</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr"/>
@@ -949,37 +949,37 @@
     <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>U-064</t>
+          <t>U-085</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C4</t>
+          <t>R1C1</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Small blue-gray circular object</t>
+          <t>Gray hexagonal emblem</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr"/>
@@ -992,37 +992,37 @@
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>U-065</t>
+          <t>U-086</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C5</t>
+          <t>R1C2</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Blue/gold polygonal plaque</t>
+          <t>Red angular object</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr"/>
@@ -1035,37 +1035,37 @@
     <row r="14" ht="42" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>U-066</t>
+          <t>U-087</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C6</t>
+          <t>R1C3</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Pale silver folded card/scroll</t>
+          <t>White curved item; a white “1” overlay is visible</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>R1C3 has visible “1”; meaning unconfirmed</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr"/>
@@ -1078,37 +1078,37 @@
     <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>U-067</t>
+          <t>U-088</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R2C7</t>
+          <t>R1C4</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Yellow-gray ornate block/emblem</t>
+          <t>Red triangle/rune-like icon</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr"/>
@@ -1121,37 +1121,37 @@
     <row r="16" ht="42" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>U-068</t>
+          <t>U-089</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C1</t>
+          <t>R2C1</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Brown oval spiral/relic icon</t>
+          <t>Gold/red plate-like icon</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr"/>
@@ -1164,37 +1164,37 @@
     <row r="17" ht="42" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>U-069</t>
+          <t>U-090</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C2</t>
+          <t>R2C2</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Dark brown/red ring-shaped relic</t>
+          <t>Red orb</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr"/>
@@ -1207,37 +1207,37 @@
     <row r="18" ht="42" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>U-070</t>
+          <t>U-091</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C3</t>
+          <t>R2C3</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Bronze-brown ring/loop icon</t>
+          <t>Blue pointed shard</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr"/>
@@ -1250,37 +1250,37 @@
     <row r="19" ht="42" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>U-071</t>
+          <t>U-092</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C4</t>
+          <t>R2C4</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Tan folded scroll/loop icon</t>
+          <t>Red hand/wing-like icon</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr"/>
@@ -1293,37 +1293,37 @@
     <row r="20" ht="42" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>U-072</t>
+          <t>U-093</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C5</t>
+          <t>R3C1</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Pale brown curved ring/relic</t>
+          <t>Blue rune/plate-like icon</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr"/>
@@ -1336,37 +1336,37 @@
     <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>U-073</t>
+          <t>U-094</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C6</t>
+          <t>R3C2</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Brown oval ring/relic</t>
+          <t>Dark red shard</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr"/>
@@ -1379,37 +1379,37 @@
     <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>U-074</t>
+          <t>U-095</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Maps, shared lower grid</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Maps Tab/Tier 1 - No Maps.PNG (same 3×7 grid repeats in Tier 1/2/3 screenshots)</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Shared lower grid R3C7</t>
+          <t>R3C3</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Brown spiral/loop relic</t>
+          <t>Flame-shaped icon</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>No number visible</t>
+          <t>No readable count</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Exact identity and whether this is inventory content or a shared UI/material grid are unknown.</t>
+          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr"/>
@@ -1422,12 +1422,12 @@
     <row r="23" ht="42" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>U-075</t>
+          <t>U-096</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -1437,12 +1437,12 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>R1C1</t>
+          <t>R3C4</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Round-headed brown wand/key-like icon</t>
+          <t>Dark framed tablet/book-like icon</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1465,12 +1465,12 @@
     <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>U-076</t>
+          <t>U-097</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -1480,12 +1480,12 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>R1C2</t>
+          <t>R4C1</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Round-headed gold wand/key-like icon</t>
+          <t>Multi-stone emblem</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1508,12 +1508,12 @@
     <row r="25" ht="42" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>U-077</t>
+          <t>U-098</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -1523,12 +1523,12 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>R1C3</t>
+          <t>R4C2</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Round-headed gray wand/key-like icon</t>
+          <t>Red orb</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1551,12 +1551,12 @@
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>U-078</t>
+          <t>U-099</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -1566,12 +1566,12 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>R2C1</t>
+          <t>R4C3</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Vertical brown key-shaped icon</t>
+          <t>Blue orb</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1594,12 +1594,12 @@
     <row r="27" ht="42" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>U-079</t>
+          <t>U-100</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Inventory — Ubers (right grid)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -1609,12 +1609,12 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>R2C2</t>
+          <t>R4C4</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Vertical gold key-shaped icon</t>
+          <t>Brown spiral/swirl icon</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1637,37 +1637,37 @@
     <row r="28" ht="42" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>U-080</t>
+          <t>U-101</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>R2C3</t>
+          <t>Top-centre crossed-axe icon</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Vertical silver key-shaped icon</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>No readable count</t>
+          <t>14 points</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Previously read as possibly Double Swing or Double Throw; confirm exact skill name.</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr"/>
@@ -1680,37 +1680,37 @@
     <row r="29" ht="42" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>U-081</t>
+          <t>U-102</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>R3C1</t>
+          <t>Upper-right node</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Brown mottled oval/organ-like icon</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>No readable count</t>
+          <t>21 points</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Skill name was not confirmed from tooltip.</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr"/>
@@ -1723,37 +1723,37 @@
     <row r="30" ht="42" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>U-082</t>
+          <t>U-103</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>R3C2</t>
+          <t>Mid-right node</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Pale circular eye-like icon with red markings</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>No readable count</t>
+          <t>21 points</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Skill name was not confirmed from tooltip.</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr"/>
@@ -1766,37 +1766,37 @@
     <row r="31" ht="42" customHeight="1">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>U-083</t>
+          <t>U-104</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Character — Combat Skills</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>R3C3</t>
+          <t>Prerequisite path / lower nodes</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Narrow pale curved/blade-like icon</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>No readable count</t>
+          <t>Several nodes show 2 points</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Prior summary did not preserve exact coordinates/names for every 2-point node; identify if useful.</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr"/>
@@ -1809,37 +1809,37 @@
     <row r="32" ht="42" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>U-084</t>
+          <t>U-105</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (left grid)</t>
+          <t>Character — Combat Masteries</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>R4C2</t>
+          <t>Top-right thrown-weapon icon</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Pale green circular medallion with geometric symbol</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>No readable count</t>
+          <t>21 points</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Previously inferred as Throw Mastery; confirm exact label.</t>
         </is>
       </c>
       <c r="H32" s="3" t="inlineStr"/>
@@ -1852,37 +1852,37 @@
     <row r="33" ht="42" customHeight="1">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>U-085</t>
+          <t>U-106</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (right grid)</t>
+          <t>Character — Combat Masteries</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>R1C1</t>
+          <t>Left-mid, right-mid, bottom-left, bottom-right nodes</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Gray hexagonal emblem</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>No readable count</t>
+          <t>2 points each</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Skill names not confirmed by hover labels.</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr"/>
@@ -1895,37 +1895,37 @@
     <row r="34" ht="42" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>U-086</t>
+          <t>U-107</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (right grid)</t>
+          <t>Character — Warcries</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>R1C2</t>
+          <t>Top-right node</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Red angular object</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>No readable count</t>
+          <t>4 points</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Previously inferred as Battle Command; confirm exact label.</t>
         </is>
       </c>
       <c r="H34" s="3" t="inlineStr"/>
@@ -1938,37 +1938,37 @@
     <row r="35" ht="42" customHeight="1">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>U-087</t>
+          <t>U-108</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Inventory — Ubers (right grid)</t>
+          <t>Character — Warcries</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
+          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>R1C3</t>
+          <t>Left-side node path</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>White curved item; a white “1” overlay is visible</t>
+          <t>Skill-tree icon; visual icon not named with confidence</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>R1C3 has visible “1”; meaning unconfirmed</t>
+          <t>Four nodes show 2 points each</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
+          <t>Previously summarized as the Battle Orders/Shout/Find Potion path; exact names/positions need confirmation.</t>
         </is>
       </c>
       <c r="H35" s="3" t="inlineStr"/>
@@ -1978,909 +1978,27 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="42" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>U-088</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>R1C4</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>Red triangle/rune-like icon</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="42" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>U-089</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>R2C1</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>Gold/red plate-like icon</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="42" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>U-090</t>
-        </is>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C38" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D38" s="2" t="inlineStr">
-        <is>
-          <t>R2C2</t>
-        </is>
-      </c>
-      <c r="E38" s="2" t="inlineStr">
-        <is>
-          <t>Red orb</t>
-        </is>
-      </c>
-      <c r="F38" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G38" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="42" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>U-091</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>R2C3</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>Blue pointed shard</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="42" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>U-092</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>R2C4</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>Red hand/wing-like icon</t>
-        </is>
-      </c>
-      <c r="F40" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H40" s="3" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="42" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>U-093</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>R3C1</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>Blue rune/plate-like icon</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="42" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>U-094</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>R3C2</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>Dark red shard</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H42" s="3" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="42" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>U-095</t>
-        </is>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C43" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>R3C3</t>
-        </is>
-      </c>
-      <c r="E43" s="2" t="inlineStr">
-        <is>
-          <t>Flame-shaped icon</t>
-        </is>
-      </c>
-      <c r="F43" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H43" s="3" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="42" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>U-096</t>
-        </is>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C44" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D44" s="2" t="inlineStr">
-        <is>
-          <t>R3C4</t>
-        </is>
-      </c>
-      <c r="E44" s="2" t="inlineStr">
-        <is>
-          <t>Dark framed tablet/book-like icon</t>
-        </is>
-      </c>
-      <c r="F44" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G44" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H44" s="3" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="42" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>U-097</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>R4C1</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>Multi-stone emblem</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H45" s="3" t="inlineStr"/>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="42" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>U-098</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>R4C2</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>Red orb</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H46" s="3" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="42" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>U-099</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>R4C3</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>Blue orb</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H47" s="3" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="42" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>U-100</t>
-        </is>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Inventory — Ubers (right grid)</t>
-        </is>
-      </c>
-      <c r="C48" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 04 - Inventory/Ubers Tab/Ubers.PNG</t>
-        </is>
-      </c>
-      <c r="D48" s="2" t="inlineStr">
-        <is>
-          <t>R4C4</t>
-        </is>
-      </c>
-      <c r="E48" s="2" t="inlineStr">
-        <is>
-          <t>Brown spiral/swirl icon</t>
-        </is>
-      </c>
-      <c r="F48" s="2" t="inlineStr">
-        <is>
-          <t>No readable count</t>
-        </is>
-      </c>
-      <c r="G48" s="2" t="inlineStr">
-        <is>
-          <t>No tooltip; exact name, quality, quantity, and tradeability unknown.</t>
-        </is>
-      </c>
-      <c r="H48" s="3" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="42" customHeight="1">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>U-101</t>
-        </is>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C49" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Top-centre crossed-axe icon</t>
-        </is>
-      </c>
-      <c r="E49" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F49" s="2" t="inlineStr">
-        <is>
-          <t>14 points</t>
-        </is>
-      </c>
-      <c r="G49" s="2" t="inlineStr">
-        <is>
-          <t>Previously read as possibly Double Swing or Double Throw; confirm exact skill name.</t>
-        </is>
-      </c>
-      <c r="H49" s="3" t="inlineStr"/>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="42" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>U-102</t>
-        </is>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C50" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D50" s="2" t="inlineStr">
-        <is>
-          <t>Upper-right node</t>
-        </is>
-      </c>
-      <c r="E50" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F50" s="2" t="inlineStr">
-        <is>
-          <t>21 points</t>
-        </is>
-      </c>
-      <c r="G50" s="2" t="inlineStr">
-        <is>
-          <t>Skill name was not confirmed from tooltip.</t>
-        </is>
-      </c>
-      <c r="H50" s="3" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="42" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>U-103</t>
-        </is>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C51" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D51" s="2" t="inlineStr">
-        <is>
-          <t>Mid-right node</t>
-        </is>
-      </c>
-      <c r="E51" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F51" s="2" t="inlineStr">
-        <is>
-          <t>21 points</t>
-        </is>
-      </c>
-      <c r="G51" s="2" t="inlineStr">
-        <is>
-          <t>Skill name was not confirmed from tooltip.</t>
-        </is>
-      </c>
-      <c r="H51" s="3" t="inlineStr"/>
-      <c r="I51" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="42" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>U-104</t>
-        </is>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Skills</t>
-        </is>
-      </c>
-      <c r="C52" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Skills.PNG</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="inlineStr">
-        <is>
-          <t>Prerequisite path / lower nodes</t>
-        </is>
-      </c>
-      <c r="E52" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F52" s="2" t="inlineStr">
-        <is>
-          <t>Several nodes show 2 points</t>
-        </is>
-      </c>
-      <c r="G52" s="2" t="inlineStr">
-        <is>
-          <t>Prior summary did not preserve exact coordinates/names for every 2-point node; identify if useful.</t>
-        </is>
-      </c>
-      <c r="H52" s="3" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="42" customHeight="1">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>U-105</t>
-        </is>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Masteries</t>
-        </is>
-      </c>
-      <c r="C53" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
-        </is>
-      </c>
-      <c r="D53" s="2" t="inlineStr">
-        <is>
-          <t>Top-right thrown-weapon icon</t>
-        </is>
-      </c>
-      <c r="E53" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F53" s="2" t="inlineStr">
-        <is>
-          <t>21 points</t>
-        </is>
-      </c>
-      <c r="G53" s="2" t="inlineStr">
-        <is>
-          <t>Previously inferred as Throw Mastery; confirm exact label.</t>
-        </is>
-      </c>
-      <c r="H53" s="3" t="inlineStr"/>
-      <c r="I53" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="42" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>U-106</t>
-        </is>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Character — Combat Masteries</t>
-        </is>
-      </c>
-      <c r="C54" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Combat Masteries.PNG</t>
-        </is>
-      </c>
-      <c r="D54" s="2" t="inlineStr">
-        <is>
-          <t>Left-mid, right-mid, bottom-left, bottom-right nodes</t>
-        </is>
-      </c>
-      <c r="E54" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F54" s="2" t="inlineStr">
-        <is>
-          <t>2 points each</t>
-        </is>
-      </c>
-      <c r="G54" s="2" t="inlineStr">
-        <is>
-          <t>Skill names not confirmed by hover labels.</t>
-        </is>
-      </c>
-      <c r="H54" s="3" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="42" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>U-107</t>
-        </is>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Character — Warcries</t>
-        </is>
-      </c>
-      <c r="C55" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
-        </is>
-      </c>
-      <c r="D55" s="2" t="inlineStr">
-        <is>
-          <t>Top-right node</t>
-        </is>
-      </c>
-      <c r="E55" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F55" s="2" t="inlineStr">
-        <is>
-          <t>4 points</t>
-        </is>
-      </c>
-      <c r="G55" s="2" t="inlineStr">
-        <is>
-          <t>Previously inferred as Battle Command; confirm exact label.</t>
-        </is>
-      </c>
-      <c r="H55" s="3" t="inlineStr"/>
-      <c r="I55" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="42" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>U-108</t>
-        </is>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Character — Warcries</t>
-        </is>
-      </c>
-      <c r="C56" s="2" t="inlineStr">
-        <is>
-          <t>MAVOmusicHC - Stats - V1.0/Images/MAVOmusicHC - 01 - Character + Skill Tree/C + Warcries.PNG</t>
-        </is>
-      </c>
-      <c r="D56" s="2" t="inlineStr">
-        <is>
-          <t>Left-side node path</t>
-        </is>
-      </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>Skill-tree icon; visual icon not named with confidence</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
-        <is>
-          <t>Four nodes show 2 points each</t>
-        </is>
-      </c>
-      <c r="G56" s="2" t="inlineStr">
-        <is>
-          <t>Previously summarized as the Battle Orders/Shout/Find Potion path; exact names/positions need confirmation.</t>
-        </is>
-      </c>
-      <c r="H56" s="3" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr">
-        <is>
-          <t>Needs player identification</t>
-        </is>
-      </c>
-    </row>
+    <row r="36" ht="42" customHeight="1"/>
+    <row r="37" ht="42" customHeight="1"/>
+    <row r="38" ht="42" customHeight="1"/>
+    <row r="39" ht="42" customHeight="1"/>
+    <row r="40" ht="42" customHeight="1"/>
+    <row r="41" ht="42" customHeight="1"/>
+    <row r="42" ht="42" customHeight="1"/>
+    <row r="43" ht="42" customHeight="1"/>
+    <row r="44" ht="42" customHeight="1"/>
+    <row r="45" ht="42" customHeight="1"/>
+    <row r="46" ht="42" customHeight="1"/>
+    <row r="47" ht="42" customHeight="1"/>
+    <row r="48" ht="42" customHeight="1"/>
+    <row r="49" ht="42" customHeight="1"/>
+    <row r="50" ht="42" customHeight="1"/>
+    <row r="51" ht="42" customHeight="1"/>
+    <row r="52" ht="42" customHeight="1"/>
+    <row r="53" ht="42" customHeight="1"/>
+    <row r="54" ht="42" customHeight="1"/>
+    <row r="55" ht="42" customHeight="1"/>
+    <row r="56" ht="42" customHeight="1"/>
     <row r="57" ht="42" customHeight="1"/>
     <row r="58" ht="42" customHeight="1"/>
     <row r="59" ht="42" customHeight="1"/>
@@ -2935,7 +2053,7 @@
     <row r="108" ht="42" customHeight="1"/>
     <row r="109" ht="42" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="A1:I56"/>
+  <autoFilter ref="A1:I35"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2993,7 +2111,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>55 unresolved rows: 47 inventory/UI icons + 8 skill-tree name checks. U-001–U-053 are resolved and recorded in source documents.</t>
+          <t>34 unresolved rows: 26 Uber-tab icons + 8 skill-tree name checks. U-001–U-074 are identified and documented.</t>
         </is>
       </c>
     </row>
@@ -3005,7 +2123,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Misc: 0; Gems bottom row: 0; Maps top tiles: 0 (names/wiki notes recorded); Maps shared lower grid: 21; Ubers: 26; skill-tree checks: 8.</t>
+          <t>Misc: 0; Gems bottom row: 0; Maps top and lower-grid icons: 0 unidentified; Ubers: 26; skill-tree checks: 8.</t>
         </is>
       </c>
     </row>
@@ -3017,7 +2135,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Top map icons are named, but the source screenshots say “No Maps” and do not confirm map ownership. The repeated lower 3×7 grid remains unidentified.</t>
+          <t>Map-tab icon names/functions are recorded in docs/04I_Inventory_Maps.md. Screenshot counts/tooltips do not establish owned quantities or saleability. Corrupted Ears U-068–U-074 are excluded from current PVM recommendations per player instruction.</t>
         </is>
       </c>
     </row>
@@ -3065,7 +2183,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Player will upload identification updates after every 20 lines. Fill “Your identification / description” for remaining rows; I will update the relevant docs and remove completed IDs from this tracker.</t>
+          <t>Player will upload identification updates after every 20 lines. Fill the remaining rows; I will update relevant docs and remove completed IDs from this tracker.</t>
         </is>
       </c>
     </row>
@@ -3089,7 +2207,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>U-001–U-015 and U-016–U-053 are resolved and documented; see docs/04D_Inventory_Misc.md, docs/04F_Inventory_Gems.md, and docs/04I_Inventory_Maps.md. Source uploads remain in docs/.</t>
+          <t>U-001–U-074 are identified and recorded in docs/04D_Inventory_Misc.md, docs/04F_Inventory_Gems.md, and docs/04I_Inventory_Maps.md. Source uploads/chat identifications are retained.</t>
         </is>
       </c>
     </row>
@@ -3101,7 +2219,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Targeted Maps page lookup completed for U-035–U-053; broader PD2 Wiki review remains deferred until all identifications are complete.</t>
+          <t>Targeted Maps Wiki lookup completed for U-025–U-067. Corrupted Ears U-068–U-074 noted as map modifiers but excluded per player scope. Broad PD2 Wiki review remains deferred until all identifications are complete.</t>
         </is>
       </c>
     </row>

</xml_diff>